<commit_message>
docs: 2FA por SMS, cadastro em etapas, celular único e sessão encerrada
- monografia (histórico 1.16): RF01, RF06, RNF12, RNF16, RN01, pacotes,
  heurísticas, sistema distribuído, componentes e resultados dos testes
- apêndice C: fluxos de cadastro em etapas, login com SMS, ativação do SMS
  e sessão encerrada ao excluir ou inativar a conta
- apêndice D: mfa_sms_phone e unicidade de phone_number no dicionário e no DER
- apêndice I: celular gateway de SMS como serviço externo
- apêndice J: casos CT39 a CT47 e bateria com 354 testes
- apêndice K: manual com o cadastro em etapas (nova Figura 1) e o MFA por SMS
</commit_message>
<xml_diff>
--- a/ApêndiceD-VisãodosDados/FalaCidade_DicionarioDados_v4.xlsx
+++ b/ApêndiceD-VisãodosDados/FalaCidade_DicionarioDados_v4.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D138"/>
+  <dimension ref="A1:D139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="D40" s="9" t="inlineStr">
         <is>
-          <t>Telefone de contato.</t>
+          <t>Telefone de contato. Único por conta (UK2): índice único pelos 11 últimos dígitos, de modo que (35) 99999-9999, 35999999999 e +55 35 99999-9999 contam como o mesmo número; telefone vazio não conta; também não pode coincidir com o celular do 2FA por SMS de outra conta (verificado na aplicação). [Fase 4]</t>
         </is>
       </c>
     </row>
@@ -1447,131 +1447,131 @@
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>mfa_sms_phone</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Data e hora de criação do registro (M).</t>
+          <t>Celular confirmado para o 2FA por SMS, no formato E.164 (ex.: +5535998761234); NULL = SMS desligado. Separado de phone_number para que a edição do telefone do perfil não redirecione o segundo fator. Único por conta (UK3, pelos 11 últimos dígitos) — RNF16. [Fase 4]</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>Data e hora de criação do registro (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
         <is>
           <t>Data e hora da última alteração (M).</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Tabela: occurrence</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>Ocorrência de zeladoria urbana registrada de forma identificada ou anônima.</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C62" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D62" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>protocol_number</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Número de protocolo exclusivo da ocorrência (UK1, M) — RF09.</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>protocol_number</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
@@ -1581,63 +1581,63 @@
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Título resumido informado pelo cidadão. [Fase 3]</t>
+          <t>Número de protocolo exclusivo da ocorrência (UK1, M) — RF09.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Descrição detalhada da ocorrência (M).</t>
+          <t>Título resumido informado pelo cidadão. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>description</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Número do imóvel de referência.</t>
+          <t>Descrição detalhada da ocorrência (M).</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>street</t>
+          <t>number</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
@@ -1647,19 +1647,19 @@
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Logradouro da ocorrência.</t>
+          <t>Número do imóvel de referência.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>neighborhood</t>
+          <t>street</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
@@ -1669,19 +1669,19 @@
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Bairro da ocorrência.</t>
+          <t>Logradouro da ocorrência.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>address_reference</t>
+          <t>neighborhood</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
@@ -1691,19 +1691,19 @@
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>100</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Ponto de referência complementar do endereço. [Fase 3]</t>
+          <t>Bairro da ocorrência.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>address_reference</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
@@ -1713,68 +1713,68 @@
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>300</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Município do endereço da ocorrência, que define a equipe responsável (M) — RF24 / RN07.</t>
+          <t>Ponto de referência complementar do endereço. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>city</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Char</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>100</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>Unidade da federação do endereço da ocorrência — RF24 / RN07. [Fase 4]</t>
+          <t>Município do endereço da ocorrência, que define a equipe responsável (M) — RF24 / RN07.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>city_id</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Char</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>FK para city — município normalizado. [Fase 3]</t>
+          <t>Unidade da federação do endereço da ocorrência — RF24 / RN07. [Fase 4]</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>city_id</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Double</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -1784,14 +1784,14 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Coordenada geográfica de latitude — RF06.</t>
+          <t>FK para city — município normalizado. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
@@ -1806,36 +1806,36 @@
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Coordenada geográfica de longitude — RF06.</t>
+          <t>Coordenada geográfica de latitude — RF06.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
         <is>
-          <t>url_media</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Double</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Endereço de entrega da primeira fotografia, já com desfoque aplicado.</t>
+          <t>Coordenada geográfica de longitude — RF06.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>cloudinary_public_id</t>
+          <t>url_media</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
@@ -1845,85 +1845,85 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>500</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Identificador público da mídia no serviço externo. [Fase 3]</t>
+          <t>Endereço de entrega da primeira fotografia, já com desfoque aplicado.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>image_blurred</t>
+          <t>cloudinary_public_id</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>255</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Indica a aplicação do desfoque de rostos e placas (M) — LGPD. [Fase 3]</t>
+          <t>Identificador público da mídia no serviço externo. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>image_blurred</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Categoria da ocorrência, conforme a enumeração OccurrenceType (M).</t>
+          <t>Indica a aplicação do desfoque de rostos e placas (M) — LGPD. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
         <is>
-          <t>classification_id</t>
+          <t>type</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>FK para classification — categoria normalizada. [Fase 3]</t>
+          <t>Categoria da ocorrência, conforme a enumeração OccurrenceType (M).</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>department_id</t>
+          <t>classification_id</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
@@ -1938,36 +1938,36 @@
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>FK para department — setor responsável pelo atendimento. [Fase 3]</t>
+          <t>FK para classification — categoria normalizada. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>department_id</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>PENDENTE, EM_ANDAMENTO, ATENDIDA ou INDEFERIDA (CK, M) — RF11.</t>
+          <t>FK para department — setor responsável pelo atendimento. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>status</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
@@ -1977,63 +1977,63 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>BAIXA, MEDIA ou ALTA (CK, M) — RF10 / RN04. [Fase 3]</t>
+          <t>PENDENTE, EM_ANDAMENTO, ATENDIDA ou INDEFERIDA (CK, M) — RF11.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
         <is>
-          <t>is_anonymous</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Indica registro sem identificação do autor (M) — RF08. [Fase 3]</t>
+          <t>BAIXA, MEDIA ou ALTA (CK, M) — RF10 / RN04. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>anonymous_tracking_code_hash</t>
+          <t>is_anonymous</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Resumo SHA-256 do código de acompanhamento anônimo — RNF17. [Fase 3]</t>
+          <t>Indica registro sem identificação do autor (M) — RF08. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>ip_address</t>
+          <t>anonymous_tracking_code_hash</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
@@ -2048,36 +2048,36 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Resumo SHA-256 do endereço de rede do autor anônimo, usado no controle do limite diário (RF08). Nunca gravado em texto claro — RNF17. [Fase 3]</t>
+          <t>Resumo SHA-256 do código de acompanhamento anônimo — RNF17. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>ip_address</t>
         </is>
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>64</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>FK para user — autor identificado da ocorrência (nulo quando anônima).</t>
+          <t>Resumo SHA-256 do endereço de rede do autor anônimo, usado no controle do limite diário (RF08). Nunca gravado em texto claro — RNF17. [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
         <is>
-          <t>group_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
@@ -2092,19 +2092,19 @@
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>FK reflexiva para occurrence — ocorrência raiz do grupo de duplicatas (RF16 / RN06). [Fase 3]</t>
+          <t>FK para user — autor identificado da ocorrência (nulo quando anônima).</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>group_id</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
@@ -2114,99 +2114,99 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Data e hora do registro da ocorrência (M).</t>
+          <t>FK reflexiva para occurrence — ocorrência raiz do grupo de duplicatas (RF16 / RN06). [Fase 3]</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
         <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D89" s="9" t="inlineStr">
+        <is>
+          <t>Data e hora do registro da ocorrência (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
+        <is>
           <t>updated_at</t>
         </is>
       </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="B90" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D89" s="9" t="inlineStr">
+      <c r="C90" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
         <is>
           <t>Data e hora da última alteração (M).</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
         <is>
           <t>Tabela: occurrence_history</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="4" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>Histórico de trâmites e mudanças de estado da ocorrência (RF11).</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="5" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B93" s="5" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C93" s="5" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D93" s="6" t="inlineStr">
+      <c r="D94" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B94" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C94" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D94" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>occurrence_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
@@ -2216,14 +2216,14 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>FK para occurrence (M).</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>changed_by</t>
+          <t>occurrence_id</t>
         </is>
       </c>
       <c r="B96" s="8" t="inlineStr">
@@ -2238,14 +2238,14 @@
       </c>
       <c r="D96" s="9" t="inlineStr">
         <is>
-          <t>FK para user — servidor responsável pela alteração.</t>
+          <t>FK para occurrence (M).</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
         <is>
-          <t>department_id</t>
+          <t>changed_by</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
@@ -2260,36 +2260,36 @@
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>FK para department — setor destinatário do encaminhamento registrado no trâmite (RF23). [Fase 4]</t>
+          <t>FK para user — servidor responsável pela alteração.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
         <is>
-          <t>old_status</t>
+          <t>department_id</t>
         </is>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
         <is>
-          <t>Estado anterior da ocorrência.</t>
+          <t>FK para department — setor destinatário do encaminhamento registrado no trâmite (RF23). [Fase 4]</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
         <is>
-          <t>new_status</t>
+          <t>old_status</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
@@ -2304,121 +2304,121 @@
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>Novo estado da ocorrência (M).</t>
+          <t>Estado anterior da ocorrência.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>observation</t>
+          <t>new_status</t>
         </is>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D100" s="9" t="inlineStr">
         <is>
-          <t>Justificativa ou observação registrada pelo servidor.</t>
+          <t>Novo estado da ocorrência (M).</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
         <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>Justificativa ou observação registrada pelo servidor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
           <t>changed_at</t>
         </is>
       </c>
-      <c r="B101" s="8" t="inlineStr">
+      <c r="B102" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C101" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D101" s="9" t="inlineStr">
+      <c r="C102" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
         <is>
           <t>Data e hora da alteração (M).</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
         <is>
           <t>Tabela: occurrence_media</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="4" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>Fotografias adicionais anexadas à ocorrência (RF07). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B105" s="5" t="inlineStr">
+      <c r="B106" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D105" s="6" t="inlineStr">
+      <c r="D106" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B106" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C106" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D106" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t>occurrence_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B107" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
@@ -2428,36 +2428,36 @@
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>FK para occurrence (M).</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>url</t>
+          <t>occurrence_id</t>
         </is>
       </c>
       <c r="B108" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
         <is>
-          <t>Endereço de entrega da imagem, já com desfoque aplicado (M).</t>
+          <t>FK para occurrence (M).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
         <is>
-          <t>cloudinary_public_id</t>
+          <t>url</t>
         </is>
       </c>
       <c r="B109" s="8" t="inlineStr">
@@ -2467,104 +2467,104 @@
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>500</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>Identificador público da mídia no serviço externo.</t>
+          <t>Endereço de entrega da imagem, já com desfoque aplicado (M).</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
+          <t>cloudinary_public_id</t>
+        </is>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>Identificador público da mídia no serviço externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="7" t="inlineStr">
+        <is>
           <t>image_blurred</t>
         </is>
       </c>
-      <c r="B110" s="8" t="inlineStr">
+      <c r="B111" s="8" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="C110" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D110" s="9" t="inlineStr">
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
         <is>
           <t>Indica a aplicação do desfoque de rostos e placas (M).</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="3" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t>Tabela: occurrence_support</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="4" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
         <is>
           <t>Reforço (apoio) de um cidadão a uma ocorrência já registrada (RF12). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="5" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B114" s="5" t="inlineStr">
+      <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C114" s="5" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr">
+      <c r="D115" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B115" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C115" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D115" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>occurrence_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B116" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
@@ -2574,14 +2574,14 @@
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>FK para occurrence (UK1 com citizen_id, M).</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>citizen_id</t>
+          <t>occurrence_id</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
@@ -2596,99 +2596,99 @@
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>FK para user — cidadão que reforçou a ocorrência (UK1 com occurrence_id).</t>
+          <t>FK para occurrence (UK1 com citizen_id, M).</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
         <is>
+          <t>citizen_id</t>
+        </is>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>FK para user — cidadão que reforçou a ocorrência (UK1 com occurrence_id).</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
           <t>supported_at</t>
         </is>
       </c>
-      <c r="B118" s="8" t="inlineStr">
+      <c r="B119" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D118" s="9" t="inlineStr">
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
         <is>
           <t>Data e hora do reforço (M).</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="3" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
         <is>
           <t>Tabela: password_reset_token</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="4" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
         <is>
           <t>Token de uso único para a redefinição de senha (RF05). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="5" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B122" s="5" t="inlineStr">
+      <c r="B123" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C122" s="5" t="inlineStr">
+      <c r="C123" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D122" s="6" t="inlineStr">
+      <c r="D123" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B123" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C123" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D123" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B124" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
@@ -2698,63 +2698,63 @@
       </c>
       <c r="D124" s="9" t="inlineStr">
         <is>
-          <t>FK para user (M).</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
         <is>
-          <t>token</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="B125" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D125" s="9" t="inlineStr">
         <is>
-          <t>Token aleatório enviado ao usuário (UK1, M).</t>
+          <t>FK para user (M).</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
         <is>
-          <t>expires_at</t>
+          <t>token</t>
         </is>
       </c>
       <c r="B126" s="8" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>255</t>
         </is>
       </c>
       <c r="D126" s="9" t="inlineStr">
         <is>
-          <t>Data e hora de expiração do token (M).</t>
+          <t>Token aleatório enviado ao usuário (UK1, M).</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
         <is>
-          <t>used</t>
+          <t>expires_at</t>
         </is>
       </c>
       <c r="B127" s="8" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Timestamp</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
@@ -2764,116 +2764,116 @@
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>Indica se o token já foi utilizado (M).</t>
+          <t>Data e hora de expiração do token (M).</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
         <is>
+          <t>used</t>
+        </is>
+      </c>
+      <c r="B128" s="8" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>Indica se o token já foi utilizado (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="7" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B128" s="8" t="inlineStr">
+      <c r="B129" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C128" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D128" s="9" t="inlineStr">
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
         <is>
           <t>Data e hora de emissão (M).</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="3" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
         <is>
           <t>Tabela: contact_message</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="4" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
         <is>
           <t>Mensagem enviada pelo formulário de contato com os administradores (RF17). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="5" t="inlineStr">
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B132" s="5" t="inlineStr">
+      <c r="B133" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C132" s="5" t="inlineStr">
+      <c r="C133" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D132" s="6" t="inlineStr">
+      <c r="D133" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B133" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C133" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D133" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B134" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D134" s="9" t="inlineStr">
         <is>
-          <t>Nome informado pelo remetente (M).</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B135" s="8" t="inlineStr">
@@ -2888,14 +2888,14 @@
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>Endereço de correio eletrônico do remetente (M).</t>
+          <t>Nome informado pelo remetente (M).</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
         <is>
-          <t>subject</t>
+          <t>email</t>
         </is>
       </c>
       <c r="B136" s="8" t="inlineStr">
@@ -2905,54 +2905,76 @@
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>150</t>
         </is>
       </c>
       <c r="D136" s="9" t="inlineStr">
         <is>
-          <t>Assunto da mensagem.</t>
+          <t>Endereço de correio eletrônico do remetente (M).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>subject</t>
         </is>
       </c>
       <c r="B137" s="8" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>255</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>Corpo da mensagem (M).</t>
+          <t>Assunto da mensagem.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
         <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="B138" s="8" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D138" s="9" t="inlineStr">
+        <is>
+          <t>Corpo da mensagem (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="7" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B138" s="8" t="inlineStr">
+      <c r="B139" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C138" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D138" s="9" t="inlineStr">
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
         <is>
           <t>Data e hora do envio (M).</t>
         </is>
@@ -2962,22 +2984,22 @@
   <mergeCells count="20">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="A92:D92"/>
+    <mergeCell ref="A132:D132"/>
+    <mergeCell ref="A113:D113"/>
+    <mergeCell ref="A122:D122"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A93:D93"/>
     <mergeCell ref="A131:D131"/>
-    <mergeCell ref="A112:D112"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="A104:D104"/>
+    <mergeCell ref="A6:D6"/>
     <mergeCell ref="A121:D121"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A130:D130"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A103:D103"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A120:D120"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A104:D104"/>
-    <mergeCell ref="A113:D113"/>
+    <mergeCell ref="A105:D105"/>
+    <mergeCell ref="A114:D114"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A32:D32"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: status Finalizada, agrupamento automático e tabela user_log
- monografia, manual, casos de teste e fluxos: exclusão lógica (Finalizada),
  agrupamento automático sem alerta, apoio como curtida e "Concluída" no lugar
  de "Atendida"; histórico mantido na versão 1.16
- apêndice D: tabela user_log no dicionário e no DER; DDL e DML do modelo
  físico atualizados
- apêndice J: bateria de 368 testes e caso CT48
</commit_message>
<xml_diff>
--- a/ApêndiceD-VisãodosDados/FalaCidade_DicionarioDados_v4.xlsx
+++ b/ApêndiceD-VisãodosDados/FalaCidade_DicionarioDados_v4.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D139"/>
+  <dimension ref="A1:D154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>PENDENTE, EM_ANDAMENTO, ATENDIDA ou INDEFERIDA (CK, M) — RF11.</t>
+          <t>PENDENTE, EM_ANDAMENTO, CONCLUIDA, INDEFERIDA ou FINALIZADA (CK, M) — RF11. FINALIZADA indica a ocorrência excluída logicamente pelo Super Administrador: situação definitiva, visível somente a esse perfil. [Fase 4]</t>
         </is>
       </c>
     </row>
@@ -2980,8 +2980,286 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>Tabela: user_log</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="4" t="inlineStr">
+        <is>
+          <t>Registro das ações da administração: criação e exclusão de contas pelo Administrador ou pelo Super Administrador e exclusão (finalização) de ocorrências pelo Super Administrador. Não copia nome nem e-mail das contas, que a consulta obtém por junção com user; conta já excluída aparece como "conta excluída". O Super Administrador vê todos os registros; o administrador municipal, somente as ações de administradores do seu município. [Fase 4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Tam.</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="7" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B144" s="8" t="inlineStr">
+        <is>
+          <t>Serial</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>Chave primária (PK).</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="B145" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>CREATE ou DELETE — criação ou exclusão da conta-alvo, ou exclusão da ocorrência (CK, M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="7" t="inlineStr">
+        <is>
+          <t>actor_id</t>
+        </is>
+      </c>
+      <c r="B146" s="8" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>FK para user — conta que executou a ação; passa a nulo se essa conta for excluída (ON DELETE SET NULL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="7" t="inlineStr">
+        <is>
+          <t>actor_role</t>
+        </is>
+      </c>
+      <c r="B147" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C147" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>Perfil de quem executou a ação no momento do registro: SUPER_ADMIN ou ADMINISTRATOR (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="7" t="inlineStr">
+        <is>
+          <t>target_id</t>
+        </is>
+      </c>
+      <c r="B148" s="8" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>FK para user — conta criada ou excluída; passa a nulo se essa conta for excluída (ON DELETE SET NULL). Nulo no registro de ocorrência excluída.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="7" t="inlineStr">
+        <is>
+          <t>target_role</t>
+        </is>
+      </c>
+      <c r="B149" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>Perfil da conta-alvo no momento do registro. Nulo no registro de ocorrência excluída.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="7" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B150" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>Município da conta-alvo ou da ocorrência excluída, usado para restringir a consulta do administrador municipal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="7" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B151" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D151" s="9" t="inlineStr">
+        <is>
+          <t>Unidade da federação correspondente a city (índice idx_user_log_locality com city).</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="7" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>Data e hora da ação (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="7" t="inlineStr">
+        <is>
+          <t>occurrence_protocol</t>
+        </is>
+      </c>
+      <c r="B153" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D153" s="9" t="inlineStr">
+        <is>
+          <t>Número de protocolo copiado da ocorrência excluída; nulo nos registros de conta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="7" t="inlineStr">
+        <is>
+          <t>occurrence_title</t>
+        </is>
+      </c>
+      <c r="B154" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>Título copiado da ocorrência excluída; nulo nos registros de conta.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A92:D92"/>
@@ -3002,6 +3280,8 @@
     <mergeCell ref="A114:D114"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A141:D141"/>
+    <mergeCell ref="A142:D142"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>

<commit_message>
docs: acesso do departamento, exclusão em cadeia, visitante com município e agrupamento a 70 m
- Monografia: RF26 (acesso do departamento e solicitação de conclusão) e RN11
  (escopo e validade do acesso); RF08, RF11, RF16, RF21, RF23 a RF25, RN01,
  RN06, RN09 e RNF17 atualizados; occurrence_history com kind e anexo; 396
  testes no back-end e 34 no front-end; linha na tabela de revisões.
- Apêndice C: fluxos de solicitação e confirmação de conclusão, entrada como
  visitante com município; encaminhamento, exclusão, mapa, máscaras e códigos.
- Apêndice D: DDL sincronizado, dicionário de dados e DER com as colunas novas.
- Apêndice I: página e API públicas do departamento e rota no Google Maps.
- Apêndice J: casos CT49 a CT67, CT23 e CT48 revistos, relatório e saídas do
  Surefire da execução de 30/09/2026.
- Apêndice K: seção do funcionário do departamento e demais perfis revistos.
- README: funcionalidades novas e como subir tudo com o subir.sh.
</commit_message>
<xml_diff>
--- a/ApêndiceD-VisãodosDados/FalaCidade_DicionarioDados_v4.xlsx
+++ b/ApêndiceD-VisãodosDados/FalaCidade_DicionarioDados_v4.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D154"/>
+  <dimension ref="A1:D157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -508,6 +508,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -610,6 +611,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -756,6 +758,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
@@ -946,6 +949,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
@@ -956,7 +960,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Usuário do sistema nos perfis Cidadão, Funcionário e Administrador.</t>
+          <t>Usuário do sistema nos perfis Cidadão, Funcionário, Administrador e Super Administrador.</t>
         </is>
       </c>
     </row>
@@ -1510,6 +1514,7 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
@@ -2162,6 +2167,7 @@
         </is>
       </c>
     </row>
+    <row r="91"/>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
@@ -2172,7 +2178,7 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Histórico de trâmites e mudanças de estado da ocorrência (RF11).</t>
+          <t>Histórico de trâmites e mudanças de estado da ocorrência (RF11) e das solicitações de conclusão enviadas pelo departamento (RF26).</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2266,7 @@
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>FK para user — servidor responsável pela alteração.</t>
+          <t>FK para user — servidor responsável pela alteração; nulo na solicitação de conclusão, feita pelo departamento sem conta no sistema.</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2354,7 @@
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>Justificativa ou observação registrada pelo servidor.</t>
+          <t>Justificativa ou observação registrada pelo servidor, ou mensagem opcional do departamento na solicitação de conclusão.</t>
         </is>
       </c>
     </row>
@@ -2374,387 +2380,390 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" s="7" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>Natureza do registro: STATUS (trâmite ou mudança de estado, valor padrão) ou COMPLETION_REQUEST (solicitação de conclusão enviada pelo departamento pelo link do encaminhamento, que não altera o estado e é visível somente à equipe) (M) — RF26. [Fase 4]</t>
+        </is>
+      </c>
+    </row>
     <row r="104">
-      <c r="A104" s="3" t="inlineStr">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>attachment_url</t>
+        </is>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>Endereço de entrega da fotografia obrigatória da solicitação de conclusão, já com desfoque aplicado; nulo nos demais registros. [Fase 4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>attachment_public_id</t>
+        </is>
+      </c>
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>Identificador público dessa fotografia no serviço externo, usado para apagá-la na exclusão da ocorrência pelo Super Administrador. [Fase 4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="106"/>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
         <is>
           <t>Tabela: occurrence_media</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="4" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
         <is>
           <t>Fotografias adicionais anexadas à ocorrência (RF07). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="5" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B106" s="5" t="inlineStr">
+      <c r="B109" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C109" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D106" s="6" t="inlineStr">
+      <c r="D109" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B107" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D107" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="7" t="inlineStr">
-        <is>
-          <t>occurrence_id</t>
-        </is>
-      </c>
-      <c r="B108" s="8" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D108" s="9" t="inlineStr">
-        <is>
-          <t>FK para occurrence (M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="B109" s="8" t="inlineStr">
-        <is>
-          <t>Varchar</t>
-        </is>
-      </c>
-      <c r="C109" s="8" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="D109" s="9" t="inlineStr">
-        <is>
-          <t>Endereço de entrega da imagem, já com desfoque aplicado (M).</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>cloudinary_public_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B110" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
         <is>
-          <t>Identificador público da mídia no serviço externo.</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
         <is>
+          <t>occurrence_id</t>
+        </is>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>FK para occurrence (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>Endereço de entrega da imagem, já com desfoque aplicado (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
+        <is>
+          <t>cloudinary_public_id</t>
+        </is>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>Identificador público da mídia no serviço externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
           <t>image_blurred</t>
         </is>
       </c>
-      <c r="B111" s="8" t="inlineStr">
+      <c r="B114" s="8" t="inlineStr">
         <is>
           <t>Boolean</t>
         </is>
       </c>
-      <c r="C111" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D111" s="9" t="inlineStr">
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
         <is>
           <t>Indica a aplicação do desfoque de rostos e placas (M).</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="3" t="inlineStr">
+    <row r="115"/>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
         <is>
           <t>Tabela: occurrence_support</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="4" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
         <is>
           <t>Reforço (apoio) de um cidadão a uma ocorrência já registrada (RF12). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="5" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B115" s="5" t="inlineStr">
+      <c r="B118" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C115" s="5" t="inlineStr">
+      <c r="C118" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D115" s="6" t="inlineStr">
+      <c r="D118" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B116" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D116" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="7" t="inlineStr">
-        <is>
-          <t>occurrence_id</t>
-        </is>
-      </c>
-      <c r="B117" s="8" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D117" s="9" t="inlineStr">
-        <is>
-          <t>FK para occurrence (UK1 com citizen_id, M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="7" t="inlineStr">
-        <is>
-          <t>citizen_id</t>
-        </is>
-      </c>
-      <c r="B118" s="8" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D118" s="9" t="inlineStr">
-        <is>
-          <t>FK para user — cidadão que reforçou a ocorrência (UK1 com occurrence_id).</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>Serial</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>Chave primária (PK).</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>occurrence_id</t>
+        </is>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>FK para occurrence (UK1 com citizen_id, M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>citizen_id</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>FK para user — cidadão que reforçou a ocorrência (UK1 com occurrence_id).</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
           <t>supported_at</t>
         </is>
       </c>
-      <c r="B119" s="8" t="inlineStr">
+      <c r="B122" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C119" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D119" s="9" t="inlineStr">
+      <c r="C122" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
         <is>
           <t>Data e hora do reforço (M).</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="3" t="inlineStr">
+    <row r="123"/>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
         <is>
           <t>Tabela: password_reset_token</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="4" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
         <is>
           <t>Token de uso único para a redefinição de senha (RF05). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="5" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B123" s="5" t="inlineStr">
+      <c r="B126" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
+      <c r="C126" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D123" s="6" t="inlineStr">
+      <c r="D126" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B124" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C124" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D124" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="7" t="inlineStr">
-        <is>
-          <t>user_id</t>
-        </is>
-      </c>
-      <c r="B125" s="8" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D125" s="9" t="inlineStr">
-        <is>
-          <t>FK para user (M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="7" t="inlineStr">
-        <is>
-          <t>token</t>
-        </is>
-      </c>
-      <c r="B126" s="8" t="inlineStr">
-        <is>
-          <t>Varchar</t>
-        </is>
-      </c>
-      <c r="C126" s="8" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="D126" s="9" t="inlineStr">
-        <is>
-          <t>Token aleatório enviado ao usuário (UK1, M).</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
         <is>
-          <t>expires_at</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B127" s="8" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
@@ -2764,19 +2773,19 @@
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>Data e hora de expiração do token (M).</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
         <is>
-          <t>used</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="B128" s="8" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
@@ -2786,372 +2795,374 @@
       </c>
       <c r="D128" s="9" t="inlineStr">
         <is>
-          <t>Indica se o token já foi utilizado (M).</t>
+          <t>FK para user (M).</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
         <is>
+          <t>token</t>
+        </is>
+      </c>
+      <c r="B129" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>Token aleatório enviado ao usuário (UK1, M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
+        <is>
+          <t>expires_at</t>
+        </is>
+      </c>
+      <c r="B130" s="8" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>Data e hora de expiração do token (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="7" t="inlineStr">
+        <is>
+          <t>used</t>
+        </is>
+      </c>
+      <c r="B131" s="8" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>Indica se o token já foi utilizado (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="7" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B129" s="8" t="inlineStr">
+      <c r="B132" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C129" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D129" s="9" t="inlineStr">
+      <c r="C132" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
         <is>
           <t>Data e hora de emissão (M).</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="3" t="inlineStr">
+    <row r="133"/>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
         <is>
           <t>Tabela: contact_message</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="4" t="inlineStr">
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
         <is>
           <t>Mensagem enviada pelo formulário de contato com os administradores (RF17). [Fase 3]</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="5" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B133" s="5" t="inlineStr">
+      <c r="B136" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C133" s="5" t="inlineStr">
+      <c r="C136" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D133" s="6" t="inlineStr">
+      <c r="D136" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B134" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C134" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D134" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="7" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B135" s="8" t="inlineStr">
-        <is>
-          <t>Varchar</t>
-        </is>
-      </c>
-      <c r="C135" s="8" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="D135" s="9" t="inlineStr">
-        <is>
-          <t>Nome informado pelo remetente (M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="7" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="B136" s="8" t="inlineStr">
-        <is>
-          <t>Varchar</t>
-        </is>
-      </c>
-      <c r="C136" s="8" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="D136" s="9" t="inlineStr">
-        <is>
-          <t>Endereço de correio eletrônico do remetente (M).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
         <is>
-          <t>subject</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B137" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t>255</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>Assunto da mensagem.</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B138" s="8" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>150</t>
         </is>
       </c>
       <c r="D138" s="9" t="inlineStr">
         <is>
-          <t>Corpo da mensagem (M).</t>
+          <t>Nome informado pelo remetente (M).</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
         <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="B139" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
+        <is>
+          <t>Endereço de correio eletrônico do remetente (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="7" t="inlineStr">
+        <is>
+          <t>subject</t>
+        </is>
+      </c>
+      <c r="B140" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C140" s="8" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>Assunto da mensagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="B141" s="8" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C141" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>Corpo da mensagem (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="7" t="inlineStr">
+        <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="B139" s="8" t="inlineStr">
+      <c r="B142" s="8" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C139" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D139" s="9" t="inlineStr">
+      <c r="C142" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
         <is>
           <t>Data e hora do envio (M).</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="A141" s="3" t="inlineStr">
+    <row r="143"/>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
         <is>
           <t>Tabela: user_log</t>
         </is>
       </c>
     </row>
-    <row r="142" ht="30" customHeight="1">
-      <c r="A142" s="4" t="inlineStr">
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
         <is>
           <t>Registro das ações da administração: criação e exclusão de contas pelo Administrador ou pelo Super Administrador e exclusão (finalização) de ocorrências pelo Super Administrador. Não copia nome nem e-mail das contas, que a consulta obtém por junção com user; conta já excluída aparece como "conta excluída". O Super Administrador vê todos os registros; o administrador municipal, somente as ações de administradores do seu município. [Fase 4]</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="5" t="inlineStr">
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
         <is>
           <t>Campo</t>
         </is>
       </c>
-      <c r="B143" s="5" t="inlineStr">
+      <c r="B146" s="5" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C143" s="5" t="inlineStr">
+      <c r="C146" s="5" t="inlineStr">
         <is>
           <t>Tam.</t>
         </is>
       </c>
-      <c r="D143" s="6" t="inlineStr">
+      <c r="D146" s="6" t="inlineStr">
         <is>
           <t>Descrição</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="7" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B144" s="8" t="inlineStr">
-        <is>
-          <t>Serial</t>
-        </is>
-      </c>
-      <c r="C144" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D144" s="9" t="inlineStr">
-        <is>
-          <t>Chave primária (PK).</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="7" t="inlineStr">
-        <is>
-          <t>action</t>
-        </is>
-      </c>
-      <c r="B145" s="8" t="inlineStr">
-        <is>
-          <t>Varchar</t>
-        </is>
-      </c>
-      <c r="C145" s="8" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D145" s="9" t="inlineStr">
-        <is>
-          <t>CREATE ou DELETE — criação ou exclusão da conta-alvo, ou exclusão da ocorrência (CK, M).</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="7" t="inlineStr">
-        <is>
-          <t>actor_id</t>
-        </is>
-      </c>
-      <c r="B146" s="8" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="C146" s="8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D146" s="9" t="inlineStr">
-        <is>
-          <t>FK para user — conta que executou a ação; passa a nulo se essa conta for excluída (ON DELETE SET NULL).</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
         <is>
-          <t>actor_role</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B147" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>Perfil de quem executou a ação no momento do registro: SUPER_ADMIN ou ADMINISTRATOR (M).</t>
+          <t>Chave primária (PK).</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
         <is>
-          <t>target_id</t>
+          <t>action</t>
         </is>
       </c>
       <c r="B148" s="8" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
         <is>
-          <t>FK para user — conta criada ou excluída; passa a nulo se essa conta for excluída (ON DELETE SET NULL). Nulo no registro de ocorrência excluída.</t>
+          <t>CREATE ou DELETE — criação ou exclusão da conta-alvo, ou exclusão da ocorrência (CK, M).</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
         <is>
-          <t>target_role</t>
+          <t>actor_id</t>
         </is>
       </c>
       <c r="B149" s="8" t="inlineStr">
         <is>
-          <t>Varchar</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C149" s="8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D149" s="9" t="inlineStr">
         <is>
-          <t>Perfil da conta-alvo no momento do registro. Nulo no registro de ocorrência excluída.</t>
+          <t>FK para user — conta que executou a ação; passa a nulo se essa conta for excluída (ON DELETE SET NULL).</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
         <is>
-          <t>city</t>
+          <t>actor_role</t>
         </is>
       </c>
       <c r="B150" s="8" t="inlineStr">
@@ -3161,63 +3172,63 @@
       </c>
       <c r="C150" s="8" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D150" s="9" t="inlineStr">
         <is>
-          <t>Município da conta-alvo ou da ocorrência excluída, usado para restringir a consulta do administrador municipal.</t>
+          <t>Perfil de quem executou a ação no momento do registro: SUPER_ADMIN ou ADMINISTRATOR (M).</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>target_id</t>
         </is>
       </c>
       <c r="B151" s="8" t="inlineStr">
         <is>
-          <t>Char</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D151" s="9" t="inlineStr">
         <is>
-          <t>Unidade da federação correspondente a city (índice idx_user_log_locality com city).</t>
+          <t>FK para user — conta criada ou excluída; passa a nulo se essa conta for excluída (ON DELETE SET NULL). Nulo no registro de ocorrência excluída.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>target_role</t>
         </is>
       </c>
       <c r="B152" s="8" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Varchar</t>
         </is>
       </c>
       <c r="C152" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D152" s="9" t="inlineStr">
         <is>
-          <t>Data e hora da ação (M).</t>
+          <t>Perfil da conta-alvo no momento do registro. Nulo no registro de ocorrência excluída.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
         <is>
-          <t>occurrence_protocol</t>
+          <t>city</t>
         </is>
       </c>
       <c r="B153" s="8" t="inlineStr">
@@ -3227,32 +3238,98 @@
       </c>
       <c r="C153" s="8" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>100</t>
         </is>
       </c>
       <c r="D153" s="9" t="inlineStr">
         <is>
-          <t>Número de protocolo copiado da ocorrência excluída; nulo nos registros de conta.</t>
+          <t>Município da conta-alvo ou da ocorrência excluída, usado para restringir a consulta do administrador municipal.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
         <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="B154" s="8" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>Unidade da federação correspondente a city (índice idx_user_log_locality com city).</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="7" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="B155" s="8" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D155" s="9" t="inlineStr">
+        <is>
+          <t>Data e hora da ação (M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="7" t="inlineStr">
+        <is>
+          <t>occurrence_protocol</t>
+        </is>
+      </c>
+      <c r="B156" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>Número de protocolo copiado da ocorrência excluída; nulo nos registros de conta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="7" t="inlineStr">
+        <is>
           <t>occurrence_title</t>
         </is>
       </c>
-      <c r="B154" s="8" t="inlineStr">
-        <is>
-          <t>Varchar</t>
-        </is>
-      </c>
-      <c r="C154" s="8" t="inlineStr">
+      <c r="B157" s="8" t="inlineStr">
+        <is>
+          <t>Varchar</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="D154" s="9" t="inlineStr">
+      <c r="D157" s="9" t="inlineStr">
         <is>
           <t>Título copiado da ocorrência excluída; nulo nos registros de conta.</t>
         </is>
@@ -3260,28 +3337,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A116:D116"/>
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A144:D144"/>
     <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A135:D135"/>
+    <mergeCell ref="A134:D134"/>
+    <mergeCell ref="A125:D125"/>
+    <mergeCell ref="A117:D117"/>
+    <mergeCell ref="A93:D93"/>
+    <mergeCell ref="A13:D13"/>
     <mergeCell ref="A92:D92"/>
-    <mergeCell ref="A132:D132"/>
-    <mergeCell ref="A113:D113"/>
-    <mergeCell ref="A122:D122"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="A93:D93"/>
-    <mergeCell ref="A131:D131"/>
+    <mergeCell ref="A107:D107"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="A61:D61"/>
-    <mergeCell ref="A104:D104"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A121:D121"/>
+    <mergeCell ref="A124:D124"/>
+    <mergeCell ref="A108:D108"/>
+    <mergeCell ref="A145:D145"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A105:D105"/>
-    <mergeCell ref="A114:D114"/>
     <mergeCell ref="A33:D33"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A141:D141"/>
-    <mergeCell ref="A142:D142"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>

</xml_diff>